<commit_message>
region map working for gas and coal capex
</commit_message>
<xml_diff>
--- a/inputs/capex_opex_converted.xlsx
+++ b/inputs/capex_opex_converted.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1091"/>
+  <dimension ref="A1:J1092"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50177,26 +50177,26 @@
         </is>
       </c>
       <c r="B1082" t="n">
-        <v>0.12</v>
+        <v>5.25</v>
       </c>
       <c r="C1082" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>World</t>
         </is>
       </c>
       <c r="D1082" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>BESS</t>
         </is>
       </c>
       <c r="E1082" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>kWh/year</t>
         </is>
       </c>
       <c r="F1082" t="inlineStr">
         <is>
-          <t>wacc</t>
+          <t>opex_f</t>
         </is>
       </c>
       <c r="G1082" t="inlineStr">
@@ -50206,17 +50206,15 @@
       </c>
       <c r="H1082" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I1082" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I1082" t="n">
+        <v>2025</v>
       </c>
       <c r="J1082" t="inlineStr">
         <is>
-          <t>IRENA 2024</t>
+          <t>Lazard 2024</t>
         </is>
       </c>
     </row>
@@ -50227,11 +50225,11 @@
         </is>
       </c>
       <c r="B1083" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="C1083" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="D1083" t="inlineStr">
@@ -50277,11 +50275,11 @@
         </is>
       </c>
       <c r="B1084" t="n">
-        <v>0.042</v>
+        <v>0.04</v>
       </c>
       <c r="C1084" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D1084" t="inlineStr">
@@ -50327,11 +50325,11 @@
         </is>
       </c>
       <c r="B1085" t="n">
-        <v>0.055</v>
+        <v>0.042</v>
       </c>
       <c r="C1085" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D1085" t="inlineStr">
@@ -50377,11 +50375,11 @@
         </is>
       </c>
       <c r="B1086" t="n">
-        <v>0.077</v>
+        <v>0.055</v>
       </c>
       <c r="C1086" t="inlineStr">
         <is>
-          <t>South America</t>
+          <t>North America</t>
         </is>
       </c>
       <c r="D1086" t="inlineStr">
@@ -50427,11 +50425,11 @@
         </is>
       </c>
       <c r="B1087" t="n">
-        <v>0.039</v>
+        <v>0.077</v>
       </c>
       <c r="C1087" t="inlineStr">
         <is>
-          <t>Oceania</t>
+          <t>South America</t>
         </is>
       </c>
       <c r="D1087" t="inlineStr">
@@ -50477,31 +50475,31 @@
         </is>
       </c>
       <c r="B1088" t="n">
-        <v>25</v>
+        <v>0.039</v>
       </c>
       <c r="C1088" t="inlineStr">
         <is>
-          <t>World</t>
+          <t>Oceania</t>
         </is>
       </c>
       <c r="D1088" t="inlineStr">
         <is>
-          <t>Gas</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="E1088" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F1088" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>wacc</t>
         </is>
       </c>
       <c r="G1088" t="inlineStr">
         <is>
-          <t>projected</t>
+          <t>historic</t>
         </is>
       </c>
       <c r="H1088" t="inlineStr">
@@ -50516,7 +50514,7 @@
       </c>
       <c r="J1088" t="inlineStr">
         <is>
-          <t>GNESTE</t>
+          <t>IRENA 2024</t>
         </is>
       </c>
     </row>
@@ -50527,7 +50525,7 @@
         </is>
       </c>
       <c r="B1089" t="n">
-        <v>0.57</v>
+        <v>25</v>
       </c>
       <c r="C1089" t="inlineStr">
         <is>
@@ -50541,12 +50539,12 @@
       </c>
       <c r="E1089" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>years</t>
         </is>
       </c>
       <c r="F1089" t="inlineStr">
         <is>
-          <t>efficiency</t>
+          <t>life</t>
         </is>
       </c>
       <c r="G1089" t="inlineStr">
@@ -50577,7 +50575,7 @@
         </is>
       </c>
       <c r="B1090" t="n">
-        <v>40</v>
+        <v>0.57</v>
       </c>
       <c r="C1090" t="inlineStr">
         <is>
@@ -50586,17 +50584,17 @@
       </c>
       <c r="D1090" t="inlineStr">
         <is>
-          <t>Coal</t>
+          <t>Gas</t>
         </is>
       </c>
       <c r="E1090" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F1090" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>efficiency</t>
         </is>
       </c>
       <c r="G1090" t="inlineStr">
@@ -50616,7 +50614,7 @@
       </c>
       <c r="J1090" t="inlineStr">
         <is>
-          <t>GNESTE [lazard/ASSET]</t>
+          <t>GNESTE</t>
         </is>
       </c>
     </row>
@@ -50627,44 +50625,94 @@
         </is>
       </c>
       <c r="B1091" t="n">
+        <v>40</v>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>Coal</t>
+        </is>
+      </c>
+      <c r="E1091" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>life</t>
+        </is>
+      </c>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>projected</t>
+        </is>
+      </c>
+      <c r="H1091" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I1091" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1091" t="inlineStr">
+        <is>
+          <t>GNESTE [lazard/ASSET]</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B1092" t="n">
         <v>0.43</v>
       </c>
-      <c r="C1091" t="inlineStr">
+      <c r="C1092" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="D1091" t="inlineStr">
+      <c r="D1092" t="inlineStr">
         <is>
           <t>Coal</t>
         </is>
       </c>
-      <c r="E1091" t="inlineStr">
+      <c r="E1092" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F1091" t="inlineStr">
+      <c r="F1092" t="inlineStr">
         <is>
           <t>efficiency</t>
         </is>
       </c>
-      <c r="G1091" t="inlineStr">
+      <c r="G1092" t="inlineStr">
         <is>
           <t>projected</t>
         </is>
       </c>
-      <c r="H1091" t="inlineStr">
+      <c r="H1092" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I1091" t="inlineStr">
+      <c r="I1092" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J1091" t="inlineStr">
+      <c r="J1092" t="inlineStr">
         <is>
           <t>GNESTE</t>
         </is>

</xml_diff>

<commit_message>
setup main improve lcoe
</commit_message>
<xml_diff>
--- a/inputs/capex_opex_converted.xlsx
+++ b/inputs/capex_opex_converted.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1277"/>
+  <dimension ref="A1:K1278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51564,7 +51564,7 @@
         </is>
       </c>
       <c r="B1088" t="n">
-        <v>5.25</v>
+        <v>0.4320000000000001</v>
       </c>
       <c r="C1088" t="inlineStr">
         <is>
@@ -51578,12 +51578,12 @@
       </c>
       <c r="E1088" t="inlineStr">
         <is>
-          <t>kWh/year</t>
+          <t>MWh</t>
         </is>
       </c>
       <c r="F1088" t="inlineStr">
         <is>
-          <t>opex_f</t>
+          <t>opex_v</t>
         </is>
       </c>
       <c r="G1088" t="inlineStr"/>
@@ -51602,7 +51602,7 @@
       </c>
       <c r="K1088" t="inlineStr">
         <is>
-          <t>Lazard 2024</t>
+          <t>Schmidt 2023</t>
         </is>
       </c>
     </row>
@@ -53444,7 +53444,7 @@
         <v>2025</v>
       </c>
       <c r="B1128" t="n">
-        <v>1.196735571358385</v>
+        <v>15.50969176402933</v>
       </c>
       <c r="C1128" t="inlineStr">
         <is>
@@ -53487,7 +53487,7 @@
         <v>2026</v>
       </c>
       <c r="B1129" t="n">
-        <v>1.285826199208117</v>
+        <v>16.66430620859269</v>
       </c>
       <c r="C1129" t="inlineStr">
         <is>
@@ -53530,7 +53530,7 @@
         <v>2027</v>
       </c>
       <c r="B1130" t="n">
-        <v>1.349791109662167</v>
+        <v>17.49329138175838</v>
       </c>
       <c r="C1130" t="inlineStr">
         <is>
@@ -53573,7 +53573,7 @@
         <v>2028</v>
       </c>
       <c r="B1131" t="n">
-        <v>1.352468055253857</v>
+        <v>17.52798459385122</v>
       </c>
       <c r="C1131" t="inlineStr">
         <is>
@@ -53616,7 +53616,7 @@
         <v>2029</v>
       </c>
       <c r="B1132" t="n">
-        <v>1.349180578211431</v>
+        <v>17.48537889478984</v>
       </c>
       <c r="C1132" t="inlineStr">
         <is>
@@ -53659,7 +53659,7 @@
         <v>2030</v>
       </c>
       <c r="B1133" t="n">
-        <v>1.350730388817146</v>
+        <v>17.50546443863306</v>
       </c>
       <c r="C1133" t="inlineStr">
         <is>
@@ -53698,11 +53698,13 @@
       <c r="K1133" t="inlineStr"/>
     </row>
     <row r="1134">
-      <c r="A1134" t="n">
-        <v>2010</v>
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
       </c>
       <c r="B1134" t="n">
-        <v>1285.7</v>
+        <v>5.4</v>
       </c>
       <c r="C1134" t="inlineStr">
         <is>
@@ -53716,12 +53718,12 @@
       </c>
       <c r="E1134" t="inlineStr">
         <is>
-          <t>kWh</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F1134" t="inlineStr">
         <is>
-          <t>capex_e</t>
+          <t>opex_f</t>
         </is>
       </c>
       <c r="G1134" t="inlineStr"/>
@@ -53740,16 +53742,16 @@
       </c>
       <c r="K1134" t="inlineStr">
         <is>
-          <t>IRENA 2024</t>
+          <t>Schmidt 2023</t>
         </is>
       </c>
     </row>
     <row r="1135">
       <c r="A1135" t="n">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="B1135" t="n">
-        <v>1065.8</v>
+        <v>1285.7</v>
       </c>
       <c r="C1135" t="inlineStr">
         <is>
@@ -53793,10 +53795,10 @@
     </row>
     <row r="1136">
       <c r="A1136" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B1136" t="n">
-        <v>1005.1</v>
+        <v>1065.8</v>
       </c>
       <c r="C1136" t="inlineStr">
         <is>
@@ -53840,10 +53842,10 @@
     </row>
     <row r="1137">
       <c r="A1137" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B1137" t="n">
-        <v>827.5</v>
+        <v>1005.1</v>
       </c>
       <c r="C1137" t="inlineStr">
         <is>
@@ -53887,10 +53889,10 @@
     </row>
     <row r="1138">
       <c r="A1138" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B1138" t="n">
-        <v>870.8</v>
+        <v>827.5</v>
       </c>
       <c r="C1138" t="inlineStr">
         <is>
@@ -53934,10 +53936,10 @@
     </row>
     <row r="1139">
       <c r="A1139" t="n">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B1139" t="n">
-        <v>772</v>
+        <v>870.8</v>
       </c>
       <c r="C1139" t="inlineStr">
         <is>
@@ -53981,10 +53983,10 @@
     </row>
     <row r="1140">
       <c r="A1140" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B1140" t="n">
-        <v>551</v>
+        <v>772</v>
       </c>
       <c r="C1140" t="inlineStr">
         <is>
@@ -54028,10 +54030,10 @@
     </row>
     <row r="1141">
       <c r="A1141" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="B1141" t="n">
-        <v>394.85</v>
+        <v>551</v>
       </c>
       <c r="C1141" t="inlineStr">
         <is>
@@ -54075,10 +54077,10 @@
     </row>
     <row r="1142">
       <c r="A1142" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="B1142" t="n">
-        <v>355.35</v>
+        <v>394.85</v>
       </c>
       <c r="C1142" t="inlineStr">
         <is>
@@ -54122,10 +54124,10 @@
     </row>
     <row r="1143">
       <c r="A1143" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="B1143" t="n">
-        <v>166.55</v>
+        <v>355.35</v>
       </c>
       <c r="C1143" t="inlineStr">
         <is>
@@ -54169,10 +54171,10 @@
     </row>
     <row r="1144">
       <c r="A1144" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B1144" t="n">
-        <v>149.95</v>
+        <v>166.55</v>
       </c>
       <c r="C1144" t="inlineStr">
         <is>
@@ -54216,10 +54218,10 @@
     </row>
     <row r="1145">
       <c r="A1145" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B1145" t="n">
-        <v>140.9</v>
+        <v>149.95</v>
       </c>
       <c r="C1145" t="inlineStr">
         <is>
@@ -54263,10 +54265,10 @@
     </row>
     <row r="1146">
       <c r="A1146" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B1146" t="n">
-        <v>178.5</v>
+        <v>140.9</v>
       </c>
       <c r="C1146" t="inlineStr">
         <is>
@@ -54310,10 +54312,10 @@
     </row>
     <row r="1147">
       <c r="A1147" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B1147" t="n">
-        <v>135.9</v>
+        <v>178.5</v>
       </c>
       <c r="C1147" t="inlineStr">
         <is>
@@ -54357,10 +54359,10 @@
     </row>
     <row r="1148">
       <c r="A1148" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B1148" t="n">
-        <v>95.8</v>
+        <v>135.9</v>
       </c>
       <c r="C1148" t="inlineStr">
         <is>
@@ -54404,10 +54406,10 @@
     </row>
     <row r="1149">
       <c r="A1149" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B1149" t="n">
-        <v>94.83232323232323</v>
+        <v>95.8</v>
       </c>
       <c r="C1149" t="inlineStr">
         <is>
@@ -54432,7 +54434,7 @@
       <c r="G1149" t="inlineStr"/>
       <c r="H1149" t="inlineStr">
         <is>
-          <t>projected</t>
+          <t>historic</t>
         </is>
       </c>
       <c r="I1149" t="inlineStr">
@@ -54443,14 +54445,18 @@
       <c r="J1149" t="n">
         <v>2025</v>
       </c>
-      <c r="K1149" t="inlineStr"/>
+      <c r="K1149" t="inlineStr">
+        <is>
+          <t>IRENA 2024</t>
+        </is>
+      </c>
     </row>
     <row r="1150">
       <c r="A1150" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B1150" t="n">
-        <v>93.90000000000001</v>
+        <v>94.83232323232323</v>
       </c>
       <c r="C1150" t="inlineStr">
         <is>
@@ -54490,10 +54496,10 @@
     </row>
     <row r="1151">
       <c r="A1151" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B1151" t="n">
-        <v>92.90000000000001</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="C1151" t="inlineStr">
         <is>
@@ -54533,10 +54539,10 @@
     </row>
     <row r="1152">
       <c r="A1152" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B1152" t="n">
-        <v>92</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="C1152" t="inlineStr">
         <is>
@@ -54576,10 +54582,10 @@
     </row>
     <row r="1153">
       <c r="A1153" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B1153" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C1153" t="inlineStr">
         <is>
@@ -54619,10 +54625,10 @@
     </row>
     <row r="1154">
       <c r="A1154" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B1154" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C1154" t="inlineStr">
         <is>
@@ -54662,10 +54668,10 @@
     </row>
     <row r="1155">
       <c r="A1155" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B1155" t="n">
-        <v>89.09999999999999</v>
+        <v>90</v>
       </c>
       <c r="C1155" t="inlineStr">
         <is>
@@ -54705,10 +54711,10 @@
     </row>
     <row r="1156">
       <c r="A1156" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B1156" t="n">
-        <v>88.09999999999999</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="C1156" t="inlineStr">
         <is>
@@ -54748,10 +54754,10 @@
     </row>
     <row r="1157">
       <c r="A1157" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B1157" t="n">
-        <v>87.59999999999999</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="C1157" t="inlineStr">
         <is>
@@ -54791,10 +54797,10 @@
     </row>
     <row r="1158">
       <c r="A1158" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B1158" t="n">
-        <v>86.7</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="C1158" t="inlineStr">
         <is>
@@ -54834,10 +54840,10 @@
     </row>
     <row r="1159">
       <c r="A1159" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B1159" t="n">
-        <v>85.7</v>
+        <v>86.7</v>
       </c>
       <c r="C1159" t="inlineStr">
         <is>
@@ -54877,10 +54883,10 @@
     </row>
     <row r="1160">
       <c r="A1160" t="n">
-        <v>2036</v>
+        <v>2035</v>
       </c>
       <c r="B1160" t="n">
-        <v>84.8</v>
+        <v>85.7</v>
       </c>
       <c r="C1160" t="inlineStr">
         <is>
@@ -54920,10 +54926,10 @@
     </row>
     <row r="1161">
       <c r="A1161" t="n">
-        <v>2037</v>
+        <v>2036</v>
       </c>
       <c r="B1161" t="n">
-        <v>83.8</v>
+        <v>84.8</v>
       </c>
       <c r="C1161" t="inlineStr">
         <is>
@@ -54963,10 +54969,10 @@
     </row>
     <row r="1162">
       <c r="A1162" t="n">
-        <v>2038</v>
+        <v>2037</v>
       </c>
       <c r="B1162" t="n">
-        <v>83.3</v>
+        <v>83.8</v>
       </c>
       <c r="C1162" t="inlineStr">
         <is>
@@ -55006,10 +55012,10 @@
     </row>
     <row r="1163">
       <c r="A1163" t="n">
-        <v>2039</v>
+        <v>2038</v>
       </c>
       <c r="B1163" t="n">
-        <v>82.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="C1163" t="inlineStr">
         <is>
@@ -55049,10 +55055,10 @@
     </row>
     <row r="1164">
       <c r="A1164" t="n">
-        <v>2040</v>
+        <v>2039</v>
       </c>
       <c r="B1164" t="n">
-        <v>81.40000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="C1164" t="inlineStr">
         <is>
@@ -55092,10 +55098,10 @@
     </row>
     <row r="1165">
       <c r="A1165" t="n">
-        <v>2041</v>
+        <v>2040</v>
       </c>
       <c r="B1165" t="n">
-        <v>80.5</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="C1165" t="inlineStr">
         <is>
@@ -55135,10 +55141,10 @@
     </row>
     <row r="1166">
       <c r="A1166" t="n">
-        <v>2042</v>
+        <v>2041</v>
       </c>
       <c r="B1166" t="n">
-        <v>80</v>
+        <v>80.5</v>
       </c>
       <c r="C1166" t="inlineStr">
         <is>
@@ -55178,10 +55184,10 @@
     </row>
     <row r="1167">
       <c r="A1167" t="n">
-        <v>2043</v>
+        <v>2042</v>
       </c>
       <c r="B1167" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C1167" t="inlineStr">
         <is>
@@ -55221,10 +55227,10 @@
     </row>
     <row r="1168">
       <c r="A1168" t="n">
-        <v>2044</v>
+        <v>2043</v>
       </c>
       <c r="B1168" t="n">
-        <v>78.09999999999999</v>
+        <v>79</v>
       </c>
       <c r="C1168" t="inlineStr">
         <is>
@@ -55264,10 +55270,10 @@
     </row>
     <row r="1169">
       <c r="A1169" t="n">
-        <v>2045</v>
+        <v>2044</v>
       </c>
       <c r="B1169" t="n">
-        <v>77.59999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="C1169" t="inlineStr">
         <is>
@@ -55307,10 +55313,10 @@
     </row>
     <row r="1170">
       <c r="A1170" t="n">
-        <v>2046</v>
+        <v>2045</v>
       </c>
       <c r="B1170" t="n">
-        <v>76.59999999999999</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C1170" t="inlineStr">
         <is>
@@ -55350,10 +55356,10 @@
     </row>
     <row r="1171">
       <c r="A1171" t="n">
-        <v>2047</v>
+        <v>2046</v>
       </c>
       <c r="B1171" t="n">
-        <v>75.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="C1171" t="inlineStr">
         <is>
@@ -55393,10 +55399,10 @@
     </row>
     <row r="1172">
       <c r="A1172" t="n">
-        <v>2048</v>
+        <v>2047</v>
       </c>
       <c r="B1172" t="n">
-        <v>75.2</v>
+        <v>75.7</v>
       </c>
       <c r="C1172" t="inlineStr">
         <is>
@@ -55436,10 +55442,10 @@
     </row>
     <row r="1173">
       <c r="A1173" t="n">
-        <v>2049</v>
+        <v>2048</v>
       </c>
       <c r="B1173" t="n">
-        <v>74.2</v>
+        <v>75.2</v>
       </c>
       <c r="C1173" t="inlineStr">
         <is>
@@ -55479,10 +55485,10 @@
     </row>
     <row r="1174">
       <c r="A1174" t="n">
-        <v>2010</v>
+        <v>2049</v>
       </c>
       <c r="B1174" t="n">
-        <v>5142.8</v>
+        <v>74.2</v>
       </c>
       <c r="C1174" t="inlineStr">
         <is>
@@ -55496,18 +55502,18 @@
       </c>
       <c r="E1174" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kWh</t>
         </is>
       </c>
       <c r="F1174" t="inlineStr">
         <is>
-          <t>capex_p</t>
+          <t>capex_e</t>
         </is>
       </c>
       <c r="G1174" t="inlineStr"/>
       <c r="H1174" t="inlineStr">
         <is>
-          <t>historic</t>
+          <t>projected</t>
         </is>
       </c>
       <c r="I1174" t="inlineStr">
@@ -55518,18 +55524,14 @@
       <c r="J1174" t="n">
         <v>2025</v>
       </c>
-      <c r="K1174" t="inlineStr">
-        <is>
-          <t>IRENA 2024</t>
-        </is>
-      </c>
+      <c r="K1174" t="inlineStr"/>
     </row>
     <row r="1175">
       <c r="A1175" t="n">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="B1175" t="n">
-        <v>4263.2</v>
+        <v>5142.8</v>
       </c>
       <c r="C1175" t="inlineStr">
         <is>
@@ -55573,10 +55575,10 @@
     </row>
     <row r="1176">
       <c r="A1176" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B1176" t="n">
-        <v>4020.4</v>
+        <v>4263.2</v>
       </c>
       <c r="C1176" t="inlineStr">
         <is>
@@ -55620,10 +55622,10 @@
     </row>
     <row r="1177">
       <c r="A1177" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B1177" t="n">
-        <v>3310</v>
+        <v>4020.4</v>
       </c>
       <c r="C1177" t="inlineStr">
         <is>
@@ -55667,10 +55669,10 @@
     </row>
     <row r="1178">
       <c r="A1178" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B1178" t="n">
-        <v>3483.2</v>
+        <v>3310</v>
       </c>
       <c r="C1178" t="inlineStr">
         <is>
@@ -55714,10 +55716,10 @@
     </row>
     <row r="1179">
       <c r="A1179" t="n">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B1179" t="n">
-        <v>3088</v>
+        <v>3483.2</v>
       </c>
       <c r="C1179" t="inlineStr">
         <is>
@@ -55761,10 +55763,10 @@
     </row>
     <row r="1180">
       <c r="A1180" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B1180" t="n">
-        <v>2204</v>
+        <v>3088</v>
       </c>
       <c r="C1180" t="inlineStr">
         <is>
@@ -55808,10 +55810,10 @@
     </row>
     <row r="1181">
       <c r="A1181" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="B1181" t="n">
-        <v>1579.4</v>
+        <v>2204</v>
       </c>
       <c r="C1181" t="inlineStr">
         <is>
@@ -55855,10 +55857,10 @@
     </row>
     <row r="1182">
       <c r="A1182" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="B1182" t="n">
-        <v>1421.4</v>
+        <v>1579.4</v>
       </c>
       <c r="C1182" t="inlineStr">
         <is>
@@ -55902,10 +55904,10 @@
     </row>
     <row r="1183">
       <c r="A1183" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="B1183" t="n">
-        <v>666.2</v>
+        <v>1421.4</v>
       </c>
       <c r="C1183" t="inlineStr">
         <is>
@@ -55949,10 +55951,10 @@
     </row>
     <row r="1184">
       <c r="A1184" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B1184" t="n">
-        <v>599.8</v>
+        <v>666.2</v>
       </c>
       <c r="C1184" t="inlineStr">
         <is>
@@ -55996,10 +55998,10 @@
     </row>
     <row r="1185">
       <c r="A1185" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B1185" t="n">
-        <v>563.6</v>
+        <v>599.8</v>
       </c>
       <c r="C1185" t="inlineStr">
         <is>
@@ -56043,10 +56045,10 @@
     </row>
     <row r="1186">
       <c r="A1186" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B1186" t="n">
-        <v>714</v>
+        <v>563.6</v>
       </c>
       <c r="C1186" t="inlineStr">
         <is>
@@ -56090,10 +56092,10 @@
     </row>
     <row r="1187">
       <c r="A1187" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B1187" t="n">
-        <v>543.6</v>
+        <v>714</v>
       </c>
       <c r="C1187" t="inlineStr">
         <is>
@@ -56137,10 +56139,10 @@
     </row>
     <row r="1188">
       <c r="A1188" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B1188" t="n">
-        <v>383.2</v>
+        <v>543.6</v>
       </c>
       <c r="C1188" t="inlineStr">
         <is>
@@ -56184,10 +56186,10 @@
     </row>
     <row r="1189">
       <c r="A1189" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B1189" t="n">
-        <v>323.6352331606217</v>
+        <v>383.2</v>
       </c>
       <c r="C1189" t="inlineStr">
         <is>
@@ -56212,7 +56214,7 @@
       <c r="G1189" t="inlineStr"/>
       <c r="H1189" t="inlineStr">
         <is>
-          <t>projected</t>
+          <t>historic</t>
         </is>
       </c>
       <c r="I1189" t="inlineStr">
@@ -56223,14 +56225,18 @@
       <c r="J1189" t="n">
         <v>2025</v>
       </c>
-      <c r="K1189" t="inlineStr"/>
+      <c r="K1189" t="inlineStr">
+        <is>
+          <t>IRENA 2024</t>
+        </is>
+      </c>
     </row>
     <row r="1190">
       <c r="A1190" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B1190" t="n">
-        <v>273.3</v>
+        <v>323.6352331606217</v>
       </c>
       <c r="C1190" t="inlineStr">
         <is>
@@ -56270,10 +56276,10 @@
     </row>
     <row r="1191">
       <c r="A1191" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B1191" t="n">
-        <v>208.8</v>
+        <v>273.3</v>
       </c>
       <c r="C1191" t="inlineStr">
         <is>
@@ -56313,10 +56319,10 @@
     </row>
     <row r="1192">
       <c r="A1192" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B1192" t="n">
-        <v>189.5</v>
+        <v>208.8</v>
       </c>
       <c r="C1192" t="inlineStr">
         <is>
@@ -56356,10 +56362,10 @@
     </row>
     <row r="1193">
       <c r="A1193" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B1193" t="n">
-        <v>176.1</v>
+        <v>189.5</v>
       </c>
       <c r="C1193" t="inlineStr">
         <is>
@@ -56399,10 +56405,10 @@
     </row>
     <row r="1194">
       <c r="A1194" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B1194" t="n">
-        <v>167.7</v>
+        <v>176.1</v>
       </c>
       <c r="C1194" t="inlineStr">
         <is>
@@ -56442,10 +56448,10 @@
     </row>
     <row r="1195">
       <c r="A1195" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B1195" t="n">
-        <v>165.2</v>
+        <v>167.7</v>
       </c>
       <c r="C1195" t="inlineStr">
         <is>
@@ -56485,10 +56491,10 @@
     </row>
     <row r="1196">
       <c r="A1196" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B1196" t="n">
-        <v>162.7</v>
+        <v>165.2</v>
       </c>
       <c r="C1196" t="inlineStr">
         <is>
@@ -56528,10 +56534,10 @@
     </row>
     <row r="1197">
       <c r="A1197" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B1197" t="n">
-        <v>158.5</v>
+        <v>162.7</v>
       </c>
       <c r="C1197" t="inlineStr">
         <is>
@@ -56571,10 +56577,10 @@
     </row>
     <row r="1198">
       <c r="A1198" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B1198" t="n">
-        <v>155.9</v>
+        <v>158.5</v>
       </c>
       <c r="C1198" t="inlineStr">
         <is>
@@ -56614,10 +56620,10 @@
     </row>
     <row r="1199">
       <c r="A1199" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B1199" t="n">
-        <v>153.4</v>
+        <v>155.9</v>
       </c>
       <c r="C1199" t="inlineStr">
         <is>
@@ -56657,10 +56663,10 @@
     </row>
     <row r="1200">
       <c r="A1200" t="n">
-        <v>2036</v>
+        <v>2035</v>
       </c>
       <c r="B1200" t="n">
-        <v>154.3</v>
+        <v>153.4</v>
       </c>
       <c r="C1200" t="inlineStr">
         <is>
@@ -56700,10 +56706,10 @@
     </row>
     <row r="1201">
       <c r="A1201" t="n">
-        <v>2037</v>
+        <v>2036</v>
       </c>
       <c r="B1201" t="n">
-        <v>155.1</v>
+        <v>154.3</v>
       </c>
       <c r="C1201" t="inlineStr">
         <is>
@@ -56743,7 +56749,7 @@
     </row>
     <row r="1202">
       <c r="A1202" t="n">
-        <v>2038</v>
+        <v>2037</v>
       </c>
       <c r="B1202" t="n">
         <v>155.1</v>
@@ -56786,10 +56792,10 @@
     </row>
     <row r="1203">
       <c r="A1203" t="n">
-        <v>2039</v>
+        <v>2038</v>
       </c>
       <c r="B1203" t="n">
-        <v>155.9</v>
+        <v>155.1</v>
       </c>
       <c r="C1203" t="inlineStr">
         <is>
@@ -56829,10 +56835,10 @@
     </row>
     <row r="1204">
       <c r="A1204" t="n">
-        <v>2040</v>
+        <v>2039</v>
       </c>
       <c r="B1204" t="n">
-        <v>156.8</v>
+        <v>155.9</v>
       </c>
       <c r="C1204" t="inlineStr">
         <is>
@@ -56872,10 +56878,10 @@
     </row>
     <row r="1205">
       <c r="A1205" t="n">
-        <v>2041</v>
+        <v>2040</v>
       </c>
       <c r="B1205" t="n">
-        <v>157.6</v>
+        <v>156.8</v>
       </c>
       <c r="C1205" t="inlineStr">
         <is>
@@ -56915,7 +56921,7 @@
     </row>
     <row r="1206">
       <c r="A1206" t="n">
-        <v>2042</v>
+        <v>2041</v>
       </c>
       <c r="B1206" t="n">
         <v>157.6</v>
@@ -56958,7 +56964,7 @@
     </row>
     <row r="1207">
       <c r="A1207" t="n">
-        <v>2043</v>
+        <v>2042</v>
       </c>
       <c r="B1207" t="n">
         <v>157.6</v>
@@ -57001,10 +57007,10 @@
     </row>
     <row r="1208">
       <c r="A1208" t="n">
-        <v>2044</v>
+        <v>2043</v>
       </c>
       <c r="B1208" t="n">
-        <v>158.5</v>
+        <v>157.6</v>
       </c>
       <c r="C1208" t="inlineStr">
         <is>
@@ -57044,10 +57050,10 @@
     </row>
     <row r="1209">
       <c r="A1209" t="n">
-        <v>2045</v>
+        <v>2044</v>
       </c>
       <c r="B1209" t="n">
-        <v>157.6</v>
+        <v>158.5</v>
       </c>
       <c r="C1209" t="inlineStr">
         <is>
@@ -57087,10 +57093,10 @@
     </row>
     <row r="1210">
       <c r="A1210" t="n">
-        <v>2046</v>
+        <v>2045</v>
       </c>
       <c r="B1210" t="n">
-        <v>158.5</v>
+        <v>157.6</v>
       </c>
       <c r="C1210" t="inlineStr">
         <is>
@@ -57130,7 +57136,7 @@
     </row>
     <row r="1211">
       <c r="A1211" t="n">
-        <v>2047</v>
+        <v>2046</v>
       </c>
       <c r="B1211" t="n">
         <v>158.5</v>
@@ -57173,10 +57179,10 @@
     </row>
     <row r="1212">
       <c r="A1212" t="n">
-        <v>2048</v>
+        <v>2047</v>
       </c>
       <c r="B1212" t="n">
-        <v>157.6</v>
+        <v>158.5</v>
       </c>
       <c r="C1212" t="inlineStr">
         <is>
@@ -57216,7 +57222,7 @@
     </row>
     <row r="1213">
       <c r="A1213" t="n">
-        <v>2049</v>
+        <v>2048</v>
       </c>
       <c r="B1213" t="n">
         <v>157.6</v>
@@ -57258,13 +57264,11 @@
       <c r="K1213" t="inlineStr"/>
     </row>
     <row r="1214">
-      <c r="A1214" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
+      <c r="A1214" t="n">
+        <v>2049</v>
       </c>
       <c r="B1214" t="n">
-        <v>5.3</v>
+        <v>157.6</v>
       </c>
       <c r="C1214" t="inlineStr">
         <is>
@@ -57278,87 +57282,85 @@
       </c>
       <c r="E1214" t="inlineStr">
         <is>
-          <t>kWh/year</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F1214" t="inlineStr">
         <is>
-          <t>opex_f</t>
+          <t>capex_p</t>
         </is>
       </c>
       <c r="G1214" t="inlineStr"/>
       <c r="H1214" t="inlineStr">
         <is>
+          <t>projected</t>
+        </is>
+      </c>
+      <c r="I1214" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J1214" t="n">
+        <v>2025</v>
+      </c>
+      <c r="K1214" t="inlineStr"/>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B1215" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>BESS</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>kWh/year</t>
+        </is>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>opex_f</t>
+        </is>
+      </c>
+      <c r="G1215" t="inlineStr"/>
+      <c r="H1215" t="inlineStr">
+        <is>
           <t>historic</t>
         </is>
       </c>
-      <c r="I1214" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J1214" t="n">
-        <v>2025</v>
-      </c>
-      <c r="K1214" t="inlineStr">
+      <c r="I1215" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J1215" t="n">
+        <v>2025</v>
+      </c>
+      <c r="K1215" t="inlineStr">
         <is>
           <t>Lazard 2024</t>
         </is>
       </c>
-    </row>
-    <row r="1215">
-      <c r="A1215" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B1215" t="n">
-        <v>85.63939393939394</v>
-      </c>
-      <c r="C1215" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-      <c r="D1215" t="inlineStr">
-        <is>
-          <t>BESS</t>
-        </is>
-      </c>
-      <c r="E1215" t="inlineStr">
-        <is>
-          <t>kWh</t>
-        </is>
-      </c>
-      <c r="F1215" t="inlineStr">
-        <is>
-          <t>capex_e</t>
-        </is>
-      </c>
-      <c r="G1215" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H1215" t="inlineStr">
-        <is>
-          <t>projected</t>
-        </is>
-      </c>
-      <c r="I1215" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J1215" t="n">
-        <v>2025</v>
-      </c>
-      <c r="K1215" t="inlineStr"/>
     </row>
     <row r="1216">
       <c r="A1216" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B1216" t="n">
-        <v>76.59999999999999</v>
+        <v>85.63939393939394</v>
       </c>
       <c r="C1216" t="inlineStr">
         <is>
@@ -57402,10 +57404,10 @@
     </row>
     <row r="1217">
       <c r="A1217" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B1217" t="n">
-        <v>64.90000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="C1217" t="inlineStr">
         <is>
@@ -57449,10 +57451,10 @@
     </row>
     <row r="1218">
       <c r="A1218" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B1218" t="n">
-        <v>61.4</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="C1218" t="inlineStr">
         <is>
@@ -57496,10 +57498,10 @@
     </row>
     <row r="1219">
       <c r="A1219" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B1219" t="n">
-        <v>58.4</v>
+        <v>61.4</v>
       </c>
       <c r="C1219" t="inlineStr">
         <is>
@@ -57543,10 +57545,10 @@
     </row>
     <row r="1220">
       <c r="A1220" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B1220" t="n">
-        <v>57.1</v>
+        <v>58.4</v>
       </c>
       <c r="C1220" t="inlineStr">
         <is>
@@ -57590,10 +57592,10 @@
     </row>
     <row r="1221">
       <c r="A1221" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B1221" t="n">
-        <v>56.2</v>
+        <v>57.1</v>
       </c>
       <c r="C1221" t="inlineStr">
         <is>
@@ -57637,10 +57639,10 @@
     </row>
     <row r="1222">
       <c r="A1222" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B1222" t="n">
-        <v>54.9</v>
+        <v>56.2</v>
       </c>
       <c r="C1222" t="inlineStr">
         <is>
@@ -57684,10 +57686,10 @@
     </row>
     <row r="1223">
       <c r="A1223" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B1223" t="n">
-        <v>54.5</v>
+        <v>54.9</v>
       </c>
       <c r="C1223" t="inlineStr">
         <is>
@@ -57731,10 +57733,10 @@
     </row>
     <row r="1224">
       <c r="A1224" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B1224" t="n">
-        <v>53.6</v>
+        <v>54.5</v>
       </c>
       <c r="C1224" t="inlineStr">
         <is>
@@ -57778,10 +57780,10 @@
     </row>
     <row r="1225">
       <c r="A1225" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B1225" t="n">
-        <v>52.8</v>
+        <v>53.6</v>
       </c>
       <c r="C1225" t="inlineStr">
         <is>
@@ -57825,7 +57827,7 @@
     </row>
     <row r="1226">
       <c r="A1226" t="n">
-        <v>2036</v>
+        <v>2035</v>
       </c>
       <c r="B1226" t="n">
         <v>52.8</v>
@@ -57872,7 +57874,7 @@
     </row>
     <row r="1227">
       <c r="A1227" t="n">
-        <v>2037</v>
+        <v>2036</v>
       </c>
       <c r="B1227" t="n">
         <v>52.8</v>
@@ -57919,7 +57921,7 @@
     </row>
     <row r="1228">
       <c r="A1228" t="n">
-        <v>2038</v>
+        <v>2037</v>
       </c>
       <c r="B1228" t="n">
         <v>52.8</v>
@@ -57966,10 +57968,10 @@
     </row>
     <row r="1229">
       <c r="A1229" t="n">
-        <v>2039</v>
+        <v>2038</v>
       </c>
       <c r="B1229" t="n">
-        <v>52.3</v>
+        <v>52.8</v>
       </c>
       <c r="C1229" t="inlineStr">
         <is>
@@ -58013,7 +58015,7 @@
     </row>
     <row r="1230">
       <c r="A1230" t="n">
-        <v>2040</v>
+        <v>2039</v>
       </c>
       <c r="B1230" t="n">
         <v>52.3</v>
@@ -58060,10 +58062,10 @@
     </row>
     <row r="1231">
       <c r="A1231" t="n">
-        <v>2041</v>
+        <v>2040</v>
       </c>
       <c r="B1231" t="n">
-        <v>51.9</v>
+        <v>52.3</v>
       </c>
       <c r="C1231" t="inlineStr">
         <is>
@@ -58107,7 +58109,7 @@
     </row>
     <row r="1232">
       <c r="A1232" t="n">
-        <v>2042</v>
+        <v>2041</v>
       </c>
       <c r="B1232" t="n">
         <v>51.9</v>
@@ -58154,7 +58156,7 @@
     </row>
     <row r="1233">
       <c r="A1233" t="n">
-        <v>2043</v>
+        <v>2042</v>
       </c>
       <c r="B1233" t="n">
         <v>51.9</v>
@@ -58201,10 +58203,10 @@
     </row>
     <row r="1234">
       <c r="A1234" t="n">
-        <v>2044</v>
+        <v>2043</v>
       </c>
       <c r="B1234" t="n">
-        <v>51.5</v>
+        <v>51.9</v>
       </c>
       <c r="C1234" t="inlineStr">
         <is>
@@ -58248,7 +58250,7 @@
     </row>
     <row r="1235">
       <c r="A1235" t="n">
-        <v>2045</v>
+        <v>2044</v>
       </c>
       <c r="B1235" t="n">
         <v>51.5</v>
@@ -58295,10 +58297,10 @@
     </row>
     <row r="1236">
       <c r="A1236" t="n">
-        <v>2046</v>
+        <v>2045</v>
       </c>
       <c r="B1236" t="n">
-        <v>51</v>
+        <v>51.5</v>
       </c>
       <c r="C1236" t="inlineStr">
         <is>
@@ -58342,10 +58344,10 @@
     </row>
     <row r="1237">
       <c r="A1237" t="n">
-        <v>2047</v>
+        <v>2046</v>
       </c>
       <c r="B1237" t="n">
-        <v>50.6</v>
+        <v>51</v>
       </c>
       <c r="C1237" t="inlineStr">
         <is>
@@ -58389,7 +58391,7 @@
     </row>
     <row r="1238">
       <c r="A1238" t="n">
-        <v>2048</v>
+        <v>2047</v>
       </c>
       <c r="B1238" t="n">
         <v>50.6</v>
@@ -58436,10 +58438,10 @@
     </row>
     <row r="1239">
       <c r="A1239" t="n">
-        <v>2049</v>
+        <v>2048</v>
       </c>
       <c r="B1239" t="n">
-        <v>50.2</v>
+        <v>50.6</v>
       </c>
       <c r="C1239" t="inlineStr">
         <is>
@@ -58483,10 +58485,10 @@
     </row>
     <row r="1240">
       <c r="A1240" t="n">
-        <v>2025</v>
+        <v>2049</v>
       </c>
       <c r="B1240" t="n">
-        <v>342.4974093264248</v>
+        <v>50.2</v>
       </c>
       <c r="C1240" t="inlineStr">
         <is>
@@ -58500,12 +58502,12 @@
       </c>
       <c r="E1240" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kWh</t>
         </is>
       </c>
       <c r="F1240" t="inlineStr">
         <is>
-          <t>capex_p</t>
+          <t>capex_e</t>
         </is>
       </c>
       <c r="G1240" t="inlineStr">
@@ -58530,10 +58532,10 @@
     </row>
     <row r="1241">
       <c r="A1241" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B1241" t="n">
-        <v>306.1</v>
+        <v>342.4974093264248</v>
       </c>
       <c r="C1241" t="inlineStr">
         <is>
@@ -58577,10 +58579,10 @@
     </row>
     <row r="1242">
       <c r="A1242" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B1242" t="n">
-        <v>260</v>
+        <v>306.1</v>
       </c>
       <c r="C1242" t="inlineStr">
         <is>
@@ -58624,10 +58626,10 @@
     </row>
     <row r="1243">
       <c r="A1243" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B1243" t="n">
-        <v>244.9</v>
+        <v>260</v>
       </c>
       <c r="C1243" t="inlineStr">
         <is>
@@ -58671,10 +58673,10 @@
     </row>
     <row r="1244">
       <c r="A1244" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B1244" t="n">
-        <v>235.1</v>
+        <v>244.9</v>
       </c>
       <c r="C1244" t="inlineStr">
         <is>
@@ -58718,10 +58720,10 @@
     </row>
     <row r="1245">
       <c r="A1245" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B1245" t="n">
-        <v>227.1</v>
+        <v>235.1</v>
       </c>
       <c r="C1245" t="inlineStr">
         <is>
@@ -58765,10 +58767,10 @@
     </row>
     <row r="1246">
       <c r="A1246" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B1246" t="n">
-        <v>224.5</v>
+        <v>227.1</v>
       </c>
       <c r="C1246" t="inlineStr">
         <is>
@@ -58812,10 +58814,10 @@
     </row>
     <row r="1247">
       <c r="A1247" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B1247" t="n">
-        <v>222.7</v>
+        <v>224.5</v>
       </c>
       <c r="C1247" t="inlineStr">
         <is>
@@ -58859,10 +58861,10 @@
     </row>
     <row r="1248">
       <c r="A1248" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B1248" t="n">
-        <v>218.3</v>
+        <v>222.7</v>
       </c>
       <c r="C1248" t="inlineStr">
         <is>
@@ -58906,10 +58908,10 @@
     </row>
     <row r="1249">
       <c r="A1249" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B1249" t="n">
-        <v>215.6</v>
+        <v>218.3</v>
       </c>
       <c r="C1249" t="inlineStr">
         <is>
@@ -58953,10 +58955,10 @@
     </row>
     <row r="1250">
       <c r="A1250" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B1250" t="n">
-        <v>213</v>
+        <v>215.6</v>
       </c>
       <c r="C1250" t="inlineStr">
         <is>
@@ -59000,10 +59002,10 @@
     </row>
     <row r="1251">
       <c r="A1251" t="n">
-        <v>2036</v>
+        <v>2035</v>
       </c>
       <c r="B1251" t="n">
-        <v>212.1</v>
+        <v>213</v>
       </c>
       <c r="C1251" t="inlineStr">
         <is>
@@ -59047,10 +59049,10 @@
     </row>
     <row r="1252">
       <c r="A1252" t="n">
-        <v>2037</v>
+        <v>2036</v>
       </c>
       <c r="B1252" t="n">
-        <v>211.2</v>
+        <v>212.1</v>
       </c>
       <c r="C1252" t="inlineStr">
         <is>
@@ -59094,10 +59096,10 @@
     </row>
     <row r="1253">
       <c r="A1253" t="n">
-        <v>2038</v>
+        <v>2037</v>
       </c>
       <c r="B1253" t="n">
-        <v>210.3</v>
+        <v>211.2</v>
       </c>
       <c r="C1253" t="inlineStr">
         <is>
@@ -59141,7 +59143,7 @@
     </row>
     <row r="1254">
       <c r="A1254" t="n">
-        <v>2039</v>
+        <v>2038</v>
       </c>
       <c r="B1254" t="n">
         <v>210.3</v>
@@ -59188,10 +59190,10 @@
     </row>
     <row r="1255">
       <c r="A1255" t="n">
-        <v>2040</v>
+        <v>2039</v>
       </c>
       <c r="B1255" t="n">
-        <v>209.4</v>
+        <v>210.3</v>
       </c>
       <c r="C1255" t="inlineStr">
         <is>
@@ -59235,7 +59237,7 @@
     </row>
     <row r="1256">
       <c r="A1256" t="n">
-        <v>2041</v>
+        <v>2040</v>
       </c>
       <c r="B1256" t="n">
         <v>209.4</v>
@@ -59282,10 +59284,10 @@
     </row>
     <row r="1257">
       <c r="A1257" t="n">
-        <v>2042</v>
+        <v>2041</v>
       </c>
       <c r="B1257" t="n">
-        <v>208.5</v>
+        <v>209.4</v>
       </c>
       <c r="C1257" t="inlineStr">
         <is>
@@ -59329,10 +59331,10 @@
     </row>
     <row r="1258">
       <c r="A1258" t="n">
-        <v>2043</v>
+        <v>2042</v>
       </c>
       <c r="B1258" t="n">
-        <v>206.7</v>
+        <v>208.5</v>
       </c>
       <c r="C1258" t="inlineStr">
         <is>
@@ -59376,7 +59378,7 @@
     </row>
     <row r="1259">
       <c r="A1259" t="n">
-        <v>2044</v>
+        <v>2043</v>
       </c>
       <c r="B1259" t="n">
         <v>206.7</v>
@@ -59423,10 +59425,10 @@
     </row>
     <row r="1260">
       <c r="A1260" t="n">
-        <v>2045</v>
+        <v>2044</v>
       </c>
       <c r="B1260" t="n">
-        <v>205</v>
+        <v>206.7</v>
       </c>
       <c r="C1260" t="inlineStr">
         <is>
@@ -59470,7 +59472,7 @@
     </row>
     <row r="1261">
       <c r="A1261" t="n">
-        <v>2046</v>
+        <v>2045</v>
       </c>
       <c r="B1261" t="n">
         <v>205</v>
@@ -59517,10 +59519,10 @@
     </row>
     <row r="1262">
       <c r="A1262" t="n">
-        <v>2047</v>
+        <v>2046</v>
       </c>
       <c r="B1262" t="n">
-        <v>204.1</v>
+        <v>205</v>
       </c>
       <c r="C1262" t="inlineStr">
         <is>
@@ -59564,10 +59566,10 @@
     </row>
     <row r="1263">
       <c r="A1263" t="n">
-        <v>2048</v>
+        <v>2047</v>
       </c>
       <c r="B1263" t="n">
-        <v>202.3</v>
+        <v>204.1</v>
       </c>
       <c r="C1263" t="inlineStr">
         <is>
@@ -59611,101 +59613,97 @@
     </row>
     <row r="1264">
       <c r="A1264" t="n">
+        <v>2048</v>
+      </c>
+      <c r="B1264" t="n">
+        <v>202.3</v>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>BESS</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F1264" t="inlineStr">
+        <is>
+          <t>capex_p</t>
+        </is>
+      </c>
+      <c r="G1264" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>projected</t>
+        </is>
+      </c>
+      <c r="I1264" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J1264" t="n">
+        <v>2025</v>
+      </c>
+      <c r="K1264" t="inlineStr"/>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="n">
         <v>2049</v>
       </c>
-      <c r="B1264" t="n">
+      <c r="B1265" t="n">
         <v>201.4</v>
       </c>
-      <c r="C1264" t="inlineStr">
+      <c r="C1265" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="D1264" t="inlineStr">
+      <c r="D1265" t="inlineStr">
         <is>
           <t>BESS</t>
         </is>
       </c>
-      <c r="E1264" t="inlineStr">
-        <is>
-          <t>kW</t>
-        </is>
-      </c>
-      <c r="F1264" t="inlineStr">
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F1265" t="inlineStr">
         <is>
           <t>capex_p</t>
         </is>
       </c>
-      <c r="G1264" t="inlineStr">
+      <c r="G1265" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H1264" t="inlineStr">
+      <c r="H1265" t="inlineStr">
         <is>
           <t>projected</t>
         </is>
       </c>
-      <c r="I1264" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J1264" t="n">
-        <v>2025</v>
-      </c>
-      <c r="K1264" t="inlineStr"/>
-    </row>
-    <row r="1265">
-      <c r="A1265" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="B1265" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="C1265" t="inlineStr">
-        <is>
-          <t>Africa</t>
-        </is>
-      </c>
-      <c r="D1265" t="inlineStr">
-        <is>
-          <t>Solar</t>
-        </is>
-      </c>
-      <c r="E1265" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="F1265" t="inlineStr">
-        <is>
-          <t>wacc</t>
-        </is>
-      </c>
-      <c r="G1265" t="inlineStr"/>
-      <c r="H1265" t="inlineStr">
-        <is>
-          <t>historic</t>
-        </is>
-      </c>
       <c r="I1265" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J1265" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K1265" t="inlineStr">
-        <is>
-          <t>IRENA 2024</t>
-        </is>
-      </c>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J1265" t="n">
+        <v>2025</v>
+      </c>
+      <c r="K1265" t="inlineStr"/>
     </row>
     <row r="1266">
       <c r="A1266" t="inlineStr">
@@ -59714,11 +59712,11 @@
         </is>
       </c>
       <c r="B1266" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="C1266" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="D1266" t="inlineStr">
@@ -59765,11 +59763,11 @@
         </is>
       </c>
       <c r="B1267" t="n">
-        <v>0.042</v>
+        <v>0.04</v>
       </c>
       <c r="C1267" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D1267" t="inlineStr">
@@ -59816,11 +59814,11 @@
         </is>
       </c>
       <c r="B1268" t="n">
-        <v>0.055</v>
+        <v>0.042</v>
       </c>
       <c r="C1268" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D1268" t="inlineStr">
@@ -59867,11 +59865,11 @@
         </is>
       </c>
       <c r="B1269" t="n">
-        <v>0.077</v>
+        <v>0.055</v>
       </c>
       <c r="C1269" t="inlineStr">
         <is>
-          <t>South America</t>
+          <t>North America</t>
         </is>
       </c>
       <c r="D1269" t="inlineStr">
@@ -59918,11 +59916,11 @@
         </is>
       </c>
       <c r="B1270" t="n">
-        <v>0.039</v>
+        <v>0.077</v>
       </c>
       <c r="C1270" t="inlineStr">
         <is>
-          <t>Oceania</t>
+          <t>South America</t>
         </is>
       </c>
       <c r="D1270" t="inlineStr">
@@ -59969,26 +59967,26 @@
         </is>
       </c>
       <c r="B1271" t="n">
-        <v>20</v>
+        <v>0.039</v>
       </c>
       <c r="C1271" t="inlineStr">
         <is>
-          <t>World</t>
+          <t>Oceania</t>
         </is>
       </c>
       <c r="D1271" t="inlineStr">
         <is>
-          <t>Gas</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="E1271" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F1271" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>wacc</t>
         </is>
       </c>
       <c r="G1271" t="inlineStr"/>
@@ -60009,7 +60007,7 @@
       </c>
       <c r="K1271" t="inlineStr">
         <is>
-          <t>Lazard 2025</t>
+          <t>IRENA 2024</t>
         </is>
       </c>
     </row>
@@ -60020,7 +60018,7 @@
         </is>
       </c>
       <c r="B1272" t="n">
-        <v>0.57</v>
+        <v>20</v>
       </c>
       <c r="C1272" t="inlineStr">
         <is>
@@ -60034,18 +60032,18 @@
       </c>
       <c r="E1272" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>years</t>
         </is>
       </c>
       <c r="F1272" t="inlineStr">
         <is>
-          <t>efficiency</t>
+          <t>life</t>
         </is>
       </c>
       <c r="G1272" t="inlineStr"/>
       <c r="H1272" t="inlineStr">
         <is>
-          <t>projected</t>
+          <t>historic</t>
         </is>
       </c>
       <c r="I1272" t="inlineStr">
@@ -60060,7 +60058,7 @@
       </c>
       <c r="K1272" t="inlineStr">
         <is>
-          <t>GNESTE</t>
+          <t>Lazard 2025</t>
         </is>
       </c>
     </row>
@@ -60071,7 +60069,7 @@
         </is>
       </c>
       <c r="B1273" t="n">
-        <v>40</v>
+        <v>0.57</v>
       </c>
       <c r="C1273" t="inlineStr">
         <is>
@@ -60080,23 +60078,23 @@
       </c>
       <c r="D1273" t="inlineStr">
         <is>
-          <t>Coal</t>
+          <t>Gas</t>
         </is>
       </c>
       <c r="E1273" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F1273" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>efficiency</t>
         </is>
       </c>
       <c r="G1273" t="inlineStr"/>
       <c r="H1273" t="inlineStr">
         <is>
-          <t>historic</t>
+          <t>projected</t>
         </is>
       </c>
       <c r="I1273" t="inlineStr">
@@ -60111,7 +60109,7 @@
       </c>
       <c r="K1273" t="inlineStr">
         <is>
-          <t>Lazard 2025</t>
+          <t>GNESTE</t>
         </is>
       </c>
     </row>
@@ -60122,7 +60120,7 @@
         </is>
       </c>
       <c r="B1274" t="n">
-        <v>0.43</v>
+        <v>40</v>
       </c>
       <c r="C1274" t="inlineStr">
         <is>
@@ -60136,18 +60134,18 @@
       </c>
       <c r="E1274" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>years</t>
         </is>
       </c>
       <c r="F1274" t="inlineStr">
         <is>
-          <t>efficiency</t>
+          <t>life</t>
         </is>
       </c>
       <c r="G1274" t="inlineStr"/>
       <c r="H1274" t="inlineStr">
         <is>
-          <t>projected</t>
+          <t>historic</t>
         </is>
       </c>
       <c r="I1274" t="inlineStr">
@@ -60162,7 +60160,7 @@
       </c>
       <c r="K1274" t="inlineStr">
         <is>
-          <t>GNESTE</t>
+          <t>Lazard 2025</t>
         </is>
       </c>
     </row>
@@ -60173,7 +60171,7 @@
         </is>
       </c>
       <c r="B1275" t="n">
-        <v>20</v>
+        <v>0.43</v>
       </c>
       <c r="C1275" t="inlineStr">
         <is>
@@ -60182,23 +60180,23 @@
       </c>
       <c r="D1275" t="inlineStr">
         <is>
-          <t>BESS</t>
+          <t>Coal</t>
         </is>
       </c>
       <c r="E1275" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F1275" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>efficiency</t>
         </is>
       </c>
       <c r="G1275" t="inlineStr"/>
       <c r="H1275" t="inlineStr">
         <is>
-          <t>historic</t>
+          <t>projected</t>
         </is>
       </c>
       <c r="I1275" t="inlineStr">
@@ -60213,7 +60211,7 @@
       </c>
       <c r="K1275" t="inlineStr">
         <is>
-          <t>Lazard 2025</t>
+          <t>GNESTE</t>
         </is>
       </c>
     </row>
@@ -60224,7 +60222,7 @@
         </is>
       </c>
       <c r="B1276" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C1276" t="inlineStr">
         <is>
@@ -60233,7 +60231,7 @@
       </c>
       <c r="D1276" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>BESS</t>
         </is>
       </c>
       <c r="E1276" t="inlineStr">
@@ -60275,7 +60273,7 @@
         </is>
       </c>
       <c r="B1277" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C1277" t="inlineStr">
         <is>
@@ -60284,7 +60282,7 @@
       </c>
       <c r="D1277" t="inlineStr">
         <is>
-          <t>Nuclear</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="E1277" t="inlineStr">
@@ -60314,6 +60312,57 @@
         </is>
       </c>
       <c r="K1277" t="inlineStr">
+        <is>
+          <t>Lazard 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B1278" t="n">
+        <v>70</v>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>Nuclear</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>life</t>
+        </is>
+      </c>
+      <c r="G1278" t="inlineStr"/>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>historic</t>
+        </is>
+      </c>
+      <c r="I1278" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1278" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1278" t="inlineStr">
         <is>
           <t>Lazard 2025</t>
         </is>

</xml_diff>